<commit_message>
add features for the excel sheet import and export
</commit_message>
<xml_diff>
--- a/public/assets/admin_products_demo.xlsx
+++ b/public/assets/admin_products_demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\eramo-multi-vendor\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24738F3-0406-4AD1-BD10-9783AD1273C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9789B5E-1579-42A1-B624-18723AF9921C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="105">
   <si>
     <t>id</t>
   </si>
@@ -147,12 +147,6 @@
     <t>VAR-BLK-123</t>
   </si>
   <si>
-    <t>VAR-WHT-123</t>
-  </si>
-  <si>
-    <t>VAR-BLU-456</t>
-  </si>
-  <si>
     <t>region_id</t>
   </si>
   <si>
@@ -325,6 +319,27 @@
   </si>
   <si>
     <t>كلمة1-كلمة2</t>
+  </si>
+  <si>
+    <t>tags_en</t>
+  </si>
+  <si>
+    <t>tags_ar</t>
+  </si>
+  <si>
+    <t>product_sku</t>
+  </si>
+  <si>
+    <t>has_discount</t>
+  </si>
+  <si>
+    <t>price_before_discount</t>
+  </si>
+  <si>
+    <t>discount_end_date</t>
+  </si>
+  <si>
+    <t>60107456+60112456</t>
   </si>
 </sst>
 </file>
@@ -687,296 +702,293 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AF3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="12" width="24.21875" customWidth="1"/>
-    <col min="13" max="21" width="24.88671875" customWidth="1"/>
-    <col min="22" max="31" width="24.21875" customWidth="1"/>
+    <col min="1" max="7" width="24.21875" customWidth="1"/>
+    <col min="8" max="18" width="24.88671875" customWidth="1"/>
+    <col min="19" max="28" width="24.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>98</v>
+      </c>
+      <c r="R1" t="s">
+        <v>99</v>
+      </c>
+      <c r="S1" t="s">
+        <v>7</v>
+      </c>
+      <c r="T1" t="s">
+        <v>8</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="AD1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="AE1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="AF1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="1" t="s">
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="V1" t="s">
-        <v>7</v>
-      </c>
-      <c r="W1" t="s">
-        <v>8</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>13</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>14</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="1">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>74</v>
+      <c r="Q2" t="s">
+        <v>96</v>
+      </c>
+      <c r="R2" t="s">
+        <v>96</v>
+      </c>
+      <c r="S2" t="s">
+        <v>25</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>77</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="V2" t="s">
-        <v>25</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>99</v>
+        <v>80</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="W2" t="s">
+        <v>96</v>
+      </c>
+      <c r="X2" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y2">
+        <v>1</v>
+      </c>
+      <c r="Z2">
+        <v>1</v>
+      </c>
+      <c r="AA2">
+        <v>1</v>
       </c>
       <c r="AB2">
         <v>1</v>
       </c>
-      <c r="AC2">
-        <v>1</v>
-      </c>
-      <c r="AD2">
-        <v>1</v>
-      </c>
-      <c r="AE2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="AC2" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE2" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="1">
-        <v>2</v>
+      <c r="AF2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3">
-        <v>5</v>
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>35</v>
       </c>
       <c r="H3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I3" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" t="s">
         <v>36</v>
       </c>
+      <c r="I3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="N3" s="1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>96</v>
+      </c>
+      <c r="R3" t="s">
+        <v>96</v>
+      </c>
+      <c r="S3" t="s">
+        <v>34</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>77</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="V3" t="s">
-        <v>34</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>99</v>
+        <v>80</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="W3" t="s">
+        <v>96</v>
+      </c>
+      <c r="X3" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y3">
+        <v>2</v>
+      </c>
+      <c r="Z3">
+        <v>3</v>
+      </c>
+      <c r="AA3">
+        <v>4</v>
       </c>
       <c r="AB3">
-        <v>2</v>
-      </c>
-      <c r="AC3">
-        <v>3</v>
-      </c>
-      <c r="AD3">
-        <v>4</v>
-      </c>
-      <c r="AE3">
         <v>2</v>
       </c>
     </row>
@@ -998,32 +1010,32 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>4</v>
+      <c r="A3" t="s">
+        <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>28</v>
@@ -1040,70 +1052,83 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="25.5546875" customWidth="1"/>
+    <col min="2" max="6" width="21.77734375" customWidth="1"/>
+    <col min="7" max="7" width="21.77734375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>100</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
+      <c r="E1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>104</v>
       </c>
       <c r="C2">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="D2">
-        <v>199.99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3">
-        <v>102</v>
+        <v>300</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>45782</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3">
+        <v>60107456</v>
       </c>
       <c r="D3">
-        <v>209.99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4">
-        <v>103</v>
-      </c>
-      <c r="D4">
-        <v>299.99</v>
+        <v>200</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3">
+        <v>300</v>
+      </c>
+      <c r="G3" s="4">
+        <v>45782</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1117,10 +1142,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>17</v>
@@ -1181,10 +1206,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -1193,10 +1218,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -1205,28 +1230,28 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -1236,40 +1261,40 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
         <v>47</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>48</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>49</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>50</v>
       </c>
-      <c r="F2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" t="s">
-        <v>52</v>
-      </c>
       <c r="H2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="N2" s="3">
         <v>45785</v>
@@ -1278,7 +1303,7 @@
         <v>45785</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>19</v>
@@ -1291,40 +1316,40 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" t="s">
         <v>53</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>54</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>55</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>56</v>
       </c>
-      <c r="F3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" t="s">
-        <v>58</v>
-      </c>
       <c r="H3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="N3" s="3">
         <v>45785</v>
@@ -1333,7 +1358,7 @@
         <v>45785</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>28</v>
@@ -1360,19 +1385,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C1" t="s">
         <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>